<commit_message>
support data list sort
</commit_message>
<xml_diff>
--- a/test/input/ray/RT结果通知单台账-1.xlsx
+++ b/test/input/ray/RT结果通知单台账-1.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4506"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26529"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\data\code\report-generator\test\input\ray\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25CA7638-D698-457E-BA8F-27BB102E9D09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18465" windowHeight="9300"/>
+    <workbookView xWindow="3072" yWindow="3072" windowWidth="23040" windowHeight="12264" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="数据库" sheetId="5" r:id="rId1"/>
@@ -18,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="69">
   <si>
     <t>委托日期</t>
   </si>
@@ -307,12 +313,16 @@
     <t>本次委托两道</t>
     <phoneticPr fontId="9" type="noConversion"/>
   </si>
+  <si>
+    <t>2024.05.30</t>
+    <phoneticPr fontId="9" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="20">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -497,60 +507,51 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="2" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -564,31 +565,31 @@
     <xf numFmtId="49" fontId="15" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="9" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="12" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="9" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="9" fontId="15" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -597,7 +598,7 @@
     <xf numFmtId="49" fontId="16" fillId="2" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
@@ -611,7 +612,7 @@
     <xf numFmtId="49" fontId="17" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -637,13 +638,13 @@
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
-    <cellStyle name="常规 2" xfId="1"/>
-    <cellStyle name="常规 2 2" xfId="5"/>
-    <cellStyle name="常规 2 3" xfId="7"/>
-    <cellStyle name="常规 2 4" xfId="3"/>
-    <cellStyle name="常规 3" xfId="4"/>
-    <cellStyle name="常规 4" xfId="6"/>
-    <cellStyle name="常规 5" xfId="2"/>
+    <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="常规 2 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
+    <cellStyle name="常规 2 3" xfId="7" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
+    <cellStyle name="常规 2 4" xfId="3" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
+    <cellStyle name="常规 3" xfId="4" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
+    <cellStyle name="常规 4" xfId="6" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
+    <cellStyle name="常规 5" xfId="2" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -653,6 +654,14 @@
       <color rgb="FFFFFF00"/>
     </mruColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -673,7 +682,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="33" name="直接箭头连接符 32"/>
+        <xdr:cNvPr id="33" name="直接箭头连接符 32">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000021000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -994,664 +1009,660 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:V29"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="24.95" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="24.9" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.625" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9" style="2"/>
-    <col min="3" max="3" width="23" style="2" customWidth="1"/>
-    <col min="4" max="4" width="23.25" style="2" customWidth="1"/>
-    <col min="5" max="5" width="5.75" style="2" customWidth="1"/>
-    <col min="6" max="6" width="8.625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="13.875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="5.875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="5.875" style="3" customWidth="1"/>
-    <col min="10" max="10" width="6.25" style="3" customWidth="1"/>
-    <col min="11" max="11" width="11.5" style="4" customWidth="1"/>
-    <col min="12" max="12" width="13.25" style="4" customWidth="1"/>
-    <col min="13" max="13" width="10" style="4" customWidth="1"/>
-    <col min="14" max="14" width="11.75" style="4" customWidth="1"/>
-    <col min="15" max="15" width="18.875" style="4" customWidth="1"/>
-    <col min="16" max="16" width="7.75" style="4" customWidth="1"/>
-    <col min="17" max="17" width="11.125" style="4" customWidth="1"/>
-    <col min="18" max="18" width="9.5" style="4" customWidth="1"/>
-    <col min="19" max="19" width="7.625" style="5" customWidth="1"/>
-    <col min="20" max="20" width="9" style="1"/>
-    <col min="21" max="21" width="16.875" style="4" customWidth="1"/>
-    <col min="22" max="22" width="9" style="1"/>
+    <col min="1" max="1" width="9.6640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="9" style="1"/>
+    <col min="3" max="3" width="23" style="1" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" style="1" customWidth="1"/>
+    <col min="5" max="5" width="5.77734375" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="5.88671875" style="1" customWidth="1"/>
+    <col min="9" max="9" width="5.88671875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="6.21875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="11.44140625" customWidth="1"/>
+    <col min="12" max="12" width="13.21875" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="11.77734375" customWidth="1"/>
+    <col min="15" max="15" width="18.88671875" customWidth="1"/>
+    <col min="16" max="16" width="7.77734375" customWidth="1"/>
+    <col min="17" max="17" width="11.109375" customWidth="1"/>
+    <col min="18" max="18" width="9.44140625" customWidth="1"/>
+    <col min="19" max="19" width="7.6640625" customWidth="1"/>
+    <col min="21" max="21" width="16.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" s="32" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A1" s="36" t="s">
+    <row r="1" spans="1:22" s="29" customFormat="1" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="33" t="s">
+      <c r="B1" s="30" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="37" t="s">
+      <c r="E1" s="34" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="37" t="s">
+      <c r="F1" s="34" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="38" t="s">
+      <c r="G1" s="35" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="39" t="s">
+      <c r="H1" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="39" t="s">
+      <c r="I1" s="36" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="40" t="s">
+      <c r="J1" s="37" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="31" t="s">
+      <c r="K1" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="L1" s="28" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="31" t="s">
+      <c r="M1" s="28" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="34" t="s">
+      <c r="N1" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="35" t="s">
+      <c r="O1" s="32" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="31" t="s">
+      <c r="P1" s="28" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="37" t="s">
+      <c r="Q1" s="34" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="37" t="s">
+      <c r="R1" s="34" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="37" t="s">
+      <c r="S1" s="34" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="37" t="s">
+      <c r="T1" s="34" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="31" t="s">
+      <c r="U1" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="37" t="s">
+      <c r="V1" s="34" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:22" ht="24.95" customHeight="1">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C2" s="21" t="s">
+      <c r="B2" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C2" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="18" t="s">
+      <c r="E2" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="F2" s="16">
+      <c r="F2" s="13">
         <v>2314</v>
       </c>
-      <c r="G2" s="28" t="s">
+      <c r="G2" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="I2" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="25">
+      <c r="J2" s="22">
         <v>0.1</v>
       </c>
-      <c r="K2" s="17" t="s">
+      <c r="K2" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L2" s="17" t="s">
+      <c r="L2" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="M2" s="26">
+      <c r="M2" s="23">
         <v>6</v>
       </c>
-      <c r="N2" s="26">
+      <c r="N2" s="23">
         <v>6</v>
       </c>
-      <c r="O2" s="20" t="s">
+      <c r="O2" s="17" t="s">
         <v>67</v>
       </c>
-      <c r="P2" s="22" t="s">
+      <c r="P2" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="Q2" s="22" t="s">
+      <c r="Q2" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="R2" s="22" t="s">
+      <c r="R2" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S2" s="22" t="s">
+      <c r="S2" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T2" s="22" t="s">
+      <c r="T2" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U2" s="12" t="s">
+      <c r="U2" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V2" s="29" t="s">
+      <c r="V2" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:22" ht="24.95" customHeight="1">
-      <c r="A3" s="17" t="s">
+    <row r="3" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="17" t="s">
+      <c r="B3" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="C3" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="16">
+      <c r="F3" s="13">
         <v>6433</v>
       </c>
-      <c r="G3" s="28" t="s">
+      <c r="G3" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="I3" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J3" s="25">
+      <c r="J3" s="22">
         <v>0.1</v>
       </c>
-      <c r="K3" s="17" t="s">
+      <c r="K3" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L3" s="17" t="s">
+      <c r="L3" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="M3" s="26">
+      <c r="M3" s="23">
         <v>6</v>
       </c>
-      <c r="N3" s="26">
+      <c r="N3" s="23">
         <v>6</v>
       </c>
-      <c r="O3" s="20"/>
-      <c r="P3" s="22" t="s">
+      <c r="O3" s="17"/>
+      <c r="P3" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="Q3" s="22" t="s">
+      <c r="Q3" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="R3" s="22" t="s">
+      <c r="R3" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S3" s="22" t="s">
+      <c r="S3" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T3" s="22" t="s">
+      <c r="T3" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U3" s="12" t="s">
+      <c r="U3" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V3" s="29" t="s">
+      <c r="V3" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:22" ht="24.95" customHeight="1">
-      <c r="A4" s="17" t="s">
+    <row r="4" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="17" t="s">
+      <c r="B4" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F4" s="16">
+      <c r="F4" s="13">
         <v>6433</v>
       </c>
-      <c r="G4" s="28" t="s">
+      <c r="G4" s="25" t="s">
         <v>35</v>
       </c>
-      <c r="H4" s="19" t="s">
+      <c r="H4" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="I4" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="J4" s="25">
+      <c r="J4" s="22">
         <v>0.1</v>
       </c>
-      <c r="K4" s="17" t="s">
+      <c r="K4" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L4" s="17" t="s">
+      <c r="L4" s="14" t="s">
         <v>36</v>
       </c>
-      <c r="M4" s="26">
+      <c r="M4" s="23">
         <v>6</v>
       </c>
-      <c r="N4" s="26">
+      <c r="N4" s="23">
         <v>6</v>
       </c>
-      <c r="O4" s="20"/>
-      <c r="P4" s="22" t="s">
+      <c r="O4" s="17"/>
+      <c r="P4" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="Q4" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="R4" s="22" t="s">
+      <c r="R4" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="S4" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T4" s="22" t="s">
+      <c r="T4" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U4" s="12" t="s">
+      <c r="U4" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V4" s="29" t="s">
+      <c r="V4" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:22" ht="24.95" customHeight="1">
-      <c r="A5" s="17" t="s">
+    <row r="5" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="21" t="s">
+      <c r="C5" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="16">
+      <c r="F5" s="13">
         <v>4938</v>
       </c>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="25" t="s">
         <v>45</v>
       </c>
-      <c r="H5" s="19" t="s">
+      <c r="H5" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="I5" s="25" t="s">
+      <c r="I5" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J5" s="25">
+      <c r="J5" s="22">
         <v>0.1</v>
       </c>
-      <c r="K5" s="17" t="s">
+      <c r="K5" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="17" t="s">
+      <c r="L5" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="26">
+      <c r="M5" s="23">
         <v>6</v>
       </c>
-      <c r="N5" s="26">
+      <c r="N5" s="23">
         <v>6</v>
       </c>
-      <c r="O5" s="20"/>
-      <c r="P5" s="22" t="s">
+      <c r="O5" s="17"/>
+      <c r="P5" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="Q5" s="22" t="s">
+      <c r="Q5" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="R5" s="22" t="s">
+      <c r="R5" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S5" s="22" t="s">
+      <c r="S5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T5" s="22" t="s">
+      <c r="T5" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U5" s="12" t="s">
+      <c r="U5" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="V5" s="29" t="s">
+      <c r="V5" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:22" s="1" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A6" s="20" t="s">
+    <row r="6" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B6" s="20" t="s">
+      <c r="B6" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="21" t="s">
+      <c r="C6" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="D6" s="22" t="s">
+      <c r="D6" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="22" t="s">
+      <c r="E6" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="30">
+      <c r="F6" s="27">
         <v>4938</v>
       </c>
-      <c r="G6" s="23" t="s">
+      <c r="G6" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="H6" s="24" t="s">
+      <c r="H6" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="I6" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="J6" s="25">
+      <c r="J6" s="22">
         <v>0.1</v>
       </c>
-      <c r="K6" s="17" t="s">
+      <c r="K6" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="17" t="s">
+      <c r="L6" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="27">
+      <c r="M6" s="24">
         <v>8</v>
       </c>
-      <c r="N6" s="27">
+      <c r="N6" s="24">
         <v>8</v>
       </c>
-      <c r="O6" s="20"/>
-      <c r="P6" s="22" t="s">
+      <c r="O6" s="17"/>
+      <c r="P6" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="Q6" s="22" t="s">
+      <c r="Q6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="R6" s="22" t="s">
+      <c r="R6" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S6" s="22" t="s">
+      <c r="S6" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T6" s="22" t="s">
+      <c r="T6" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U6" s="12" t="s">
+      <c r="U6" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="V6" s="29" t="s">
+      <c r="V6" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:22" s="1" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A7" s="20" t="s">
+    <row r="7" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="B7" s="20" t="s">
+      <c r="B7" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="21" t="s">
+      <c r="C7" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="D7" s="22" t="s">
+      <c r="D7" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="19" t="s">
         <v>50</v>
       </c>
-      <c r="F7" s="30">
+      <c r="F7" s="27">
         <v>4938</v>
       </c>
-      <c r="G7" s="23" t="s">
+      <c r="G7" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="H7" s="24" t="s">
+      <c r="H7" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I7" s="25" t="s">
+      <c r="I7" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J7" s="25">
+      <c r="J7" s="22">
         <v>0.1</v>
       </c>
-      <c r="K7" s="17" t="s">
+      <c r="K7" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="17" t="s">
+      <c r="L7" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="M7" s="27">
+      <c r="M7" s="24">
         <v>2</v>
       </c>
-      <c r="N7" s="27">
+      <c r="N7" s="24">
         <v>1</v>
       </c>
-      <c r="O7" s="20"/>
-      <c r="P7" s="22" t="s">
+      <c r="O7" s="17"/>
+      <c r="P7" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="Q7" s="22" t="s">
+      <c r="Q7" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="R7" s="22" t="s">
+      <c r="R7" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S7" s="22" t="s">
+      <c r="S7" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T7" s="22" t="s">
+      <c r="T7" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U7" s="12" t="s">
+      <c r="U7" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="V7" s="29" t="s">
+      <c r="V7" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:22" s="1" customFormat="1" ht="24.95" customHeight="1">
-      <c r="A8" s="20" t="s">
+    <row r="8" spans="1:22" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B8" s="20" t="s">
+      <c r="B8" s="17" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="21" t="s">
+      <c r="C8" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="19" t="s">
         <v>28</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="E8" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="F8" s="30">
+      <c r="F8" s="27">
         <v>4938</v>
       </c>
-      <c r="G8" s="23" t="s">
+      <c r="G8" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="H8" s="24" t="s">
+      <c r="H8" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="I8" s="25" t="s">
+      <c r="I8" s="22" t="s">
         <v>55</v>
       </c>
-      <c r="J8" s="25">
+      <c r="J8" s="22">
         <v>0.1</v>
       </c>
-      <c r="K8" s="17" t="s">
+      <c r="K8" s="14" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="17" t="s">
+      <c r="L8" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="M8" s="27">
+      <c r="M8" s="24">
         <v>1</v>
       </c>
-      <c r="N8" s="27">
+      <c r="N8" s="24">
         <v>1</v>
       </c>
-      <c r="O8" s="20"/>
-      <c r="P8" s="22" t="s">
+      <c r="O8" s="17"/>
+      <c r="P8" s="19" t="s">
         <v>49</v>
       </c>
-      <c r="Q8" s="22" t="s">
+      <c r="Q8" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="R8" s="22" t="s">
+      <c r="R8" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="S8" s="22" t="s">
+      <c r="S8" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="T8" s="22" t="s">
+      <c r="T8" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="U8" s="12" t="s">
+      <c r="U8" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="V8" s="29" t="s">
+      <c r="V8" s="26" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:22" s="1" customFormat="1" ht="24.95" hidden="1" customHeight="1">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="9"/>
-      <c r="F9" s="9"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="11"/>
-      <c r="I9" s="25" t="s">
+    <row r="9" spans="1:22" ht="24.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="7"/>
+      <c r="H9" s="8"/>
+      <c r="I9" s="22" t="s">
         <v>54</v>
       </c>
-      <c r="J9" s="13"/>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="7"/>
-      <c r="N9" s="7"/>
-      <c r="O9" s="7"/>
-      <c r="P9" s="12"/>
-      <c r="Q9" s="12"/>
-      <c r="R9" s="12"/>
-      <c r="S9" s="15"/>
-      <c r="T9" s="15"/>
-      <c r="U9" s="12"/>
-      <c r="V9" s="15"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="4"/>
+      <c r="L9" s="4"/>
+      <c r="M9" s="4"/>
+      <c r="N9" s="4"/>
+      <c r="O9" s="4"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="12"/>
+      <c r="T9" s="12"/>
+      <c r="U9" s="9"/>
+      <c r="V9" s="12"/>
     </row>
-    <row r="10" spans="1:22" s="1" customFormat="1" ht="24.95" hidden="1" customHeight="1">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="9"/>
-      <c r="F10" s="9"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="11"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="13"/>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="7"/>
-      <c r="N10" s="7"/>
-      <c r="O10" s="7"/>
-      <c r="P10" s="12"/>
-      <c r="Q10" s="12"/>
-      <c r="R10" s="12"/>
-      <c r="S10" s="15"/>
-      <c r="T10" s="15"/>
-      <c r="U10" s="12"/>
-      <c r="V10" s="15"/>
+    <row r="10" spans="1:22" ht="24.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4"/>
+      <c r="B10" s="4"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="7"/>
+      <c r="H10" s="8"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="4"/>
+      <c r="L10" s="4"/>
+      <c r="M10" s="4"/>
+      <c r="N10" s="4"/>
+      <c r="O10" s="4"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="12"/>
+      <c r="T10" s="12"/>
+      <c r="U10" s="9"/>
+      <c r="V10" s="12"/>
     </row>
-    <row r="11" spans="1:22" s="1" customFormat="1" ht="24.95" hidden="1" customHeight="1">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="11"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="13"/>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
-      <c r="N11" s="7"/>
-      <c r="O11" s="7"/>
-      <c r="P11" s="12"/>
-      <c r="Q11" s="12"/>
-      <c r="R11" s="12"/>
-      <c r="S11" s="15"/>
-      <c r="T11" s="15"/>
-      <c r="U11" s="12"/>
-      <c r="V11" s="15"/>
+    <row r="11" spans="1:22" ht="24.9" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="7"/>
+      <c r="H11" s="8"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="10"/>
+      <c r="K11" s="4"/>
+      <c r="L11" s="4"/>
+      <c r="M11" s="4"/>
+      <c r="N11" s="4"/>
+      <c r="O11" s="4"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="12"/>
+      <c r="T11" s="12"/>
+      <c r="U11" s="9"/>
+      <c r="V11" s="12"/>
     </row>
-    <row r="25" spans="4:15" ht="24.95" customHeight="1">
-      <c r="D25" s="2" t="s">
+    <row r="25" spans="4:15" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D25" s="1" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="4:15" ht="24.95" customHeight="1">
-      <c r="D26" s="2" t="s">
+    <row r="26" spans="4:15" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D26" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="4:15" ht="24.95" customHeight="1">
-      <c r="D27" s="2" t="s">
+    <row r="27" spans="4:15" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="D27" s="1" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="4:15" ht="24.95" customHeight="1">
-      <c r="O29" s="4" t="s">
+    <row r="29" spans="4:15" ht="24.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="O29" t="s">
         <v>33</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S11">
-    <extLst/>
-  </autoFilter>
+  <autoFilter ref="A1:S11" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.118055555555556" top="0.43263888888888902" bottom="0.35416666666666702" header="0.156944444444444" footer="0.118055555555556"/>
   <pageSetup paperSize="9" scale="25" orientation="landscape" r:id="rId1"/>

</xml_diff>